<commit_message>
Update Modelo Planilha de Projecao.xlsx
</commit_message>
<xml_diff>
--- a/Modelo Planilha de Projecao.xlsx
+++ b/Modelo Planilha de Projecao.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\msj\Documents\GitHub\pyToScriptCAD\in\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\msj\Documents\GitHub\pyToScriptCAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24CC0BA2-4256-4BF2-91B9-0330DAA28543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B9F89DA-0805-4E7E-B620-D5F7A6B87FF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="831" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -776,33 +776,33 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:V179"/>
-  <sheetFormatPr defaultColWidth="3.88671875" defaultRowHeight="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="3.85546875" defaultRowHeight="13.9" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.6640625" style="11" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" style="9" customWidth="1"/>
-    <col min="3" max="3" width="2.77734375" style="5" customWidth="1"/>
-    <col min="4" max="4" width="6.33203125" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="2.77734375" style="5" customWidth="1"/>
-    <col min="10" max="10" width="24.21875" style="15" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.21875" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.5546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.7109375" style="11" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" style="9" customWidth="1"/>
+    <col min="3" max="3" width="2.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="6.28515625" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="2.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="24.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.28515625" style="7" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="19" style="7" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="2.6640625" style="27" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.6640625" style="27" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="5.6640625" style="28" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.44140625" style="28" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.33203125" style="28" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="2.6640625" style="27" bestFit="1" customWidth="1"/>
-    <col min="23" max="16384" width="3.88671875" style="5"/>
+    <col min="17" max="17" width="2.7109375" style="27" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.7109375" style="27" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5.7109375" style="28" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.42578125" style="28" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.28515625" style="28" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="2.7109375" style="27" bestFit="1" customWidth="1"/>
+    <col min="23" max="16384" width="3.85546875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="10" customFormat="1" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" s="10" customFormat="1" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
@@ -860,7 +860,7 @@
       </c>
       <c r="V1" s="22"/>
     </row>
-    <row r="2" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
         <v>60</v>
       </c>
@@ -916,7 +916,7 @@
       <c r="U2" s="24"/>
       <c r="V2" s="25"/>
     </row>
-    <row r="3" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="17" t="s">
         <v>61</v>
       </c>
@@ -972,7 +972,7 @@
       <c r="U3" s="24"/>
       <c r="V3" s="25"/>
     </row>
-    <row r="4" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="17"/>
       <c r="B4" s="19"/>
       <c r="C4" s="4"/>
@@ -1020,7 +1020,7 @@
       <c r="U4" s="24"/>
       <c r="V4" s="25"/>
     </row>
-    <row r="5" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="17"/>
       <c r="B5" s="19"/>
       <c r="C5" s="4"/>
@@ -1068,7 +1068,7 @@
       <c r="U5" s="24"/>
       <c r="V5" s="25"/>
     </row>
-    <row r="6" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="17"/>
       <c r="B6" s="18"/>
       <c r="C6" s="4"/>
@@ -1116,7 +1116,7 @@
       <c r="U6" s="24"/>
       <c r="V6" s="25"/>
     </row>
-    <row r="7" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="18"/>
       <c r="C7" s="4"/>
@@ -1154,7 +1154,7 @@
       <c r="U7" s="24"/>
       <c r="V7" s="25"/>
     </row>
-    <row r="8" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="18"/>
       <c r="C8" s="4"/>
@@ -1192,7 +1192,7 @@
       <c r="U8" s="24"/>
       <c r="V8" s="25"/>
     </row>
-    <row r="9" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="17"/>
       <c r="B9" s="18"/>
       <c r="C9" s="4"/>
@@ -1230,7 +1230,7 @@
       <c r="U9" s="24"/>
       <c r="V9" s="25"/>
     </row>
-    <row r="10" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="8"/>
       <c r="B10" s="6"/>
       <c r="C10" s="4"/>
@@ -1268,7 +1268,7 @@
       <c r="U10" s="24"/>
       <c r="V10" s="25"/>
     </row>
-    <row r="11" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="8"/>
       <c r="B11" s="6"/>
       <c r="C11" s="4"/>
@@ -1306,7 +1306,7 @@
       <c r="U11" s="24"/>
       <c r="V11" s="25"/>
     </row>
-    <row r="12" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="8"/>
       <c r="B12" s="6"/>
       <c r="C12" s="4"/>
@@ -1344,7 +1344,7 @@
       <c r="U12" s="24"/>
       <c r="V12" s="25"/>
     </row>
-    <row r="13" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="8"/>
       <c r="B13" s="6"/>
       <c r="C13" s="4"/>
@@ -1382,7 +1382,7 @@
       <c r="U13" s="24"/>
       <c r="V13" s="25"/>
     </row>
-    <row r="14" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="8"/>
       <c r="B14" s="6"/>
       <c r="C14" s="4"/>
@@ -1420,7 +1420,7 @@
       <c r="U14" s="24"/>
       <c r="V14" s="25"/>
     </row>
-    <row r="15" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="8"/>
       <c r="B15" s="6"/>
       <c r="C15" s="4"/>
@@ -1458,7 +1458,7 @@
       <c r="U15" s="24"/>
       <c r="V15" s="25"/>
     </row>
-    <row r="16" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="8"/>
       <c r="B16" s="6"/>
       <c r="C16" s="4"/>
@@ -1496,7 +1496,7 @@
       <c r="U16" s="24"/>
       <c r="V16" s="25"/>
     </row>
-    <row r="17" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="8"/>
       <c r="B17" s="6"/>
       <c r="C17" s="4"/>
@@ -1534,7 +1534,7 @@
       <c r="U17" s="24"/>
       <c r="V17" s="25"/>
     </row>
-    <row r="18" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="8"/>
       <c r="B18" s="6"/>
       <c r="C18" s="4"/>
@@ -1572,7 +1572,7 @@
       <c r="U18" s="24"/>
       <c r="V18" s="25"/>
     </row>
-    <row r="19" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="8"/>
       <c r="B19" s="6"/>
       <c r="C19" s="4"/>
@@ -1610,7 +1610,7 @@
       <c r="U19" s="26"/>
       <c r="V19" s="25"/>
     </row>
-    <row r="20" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="8"/>
       <c r="B20" s="6"/>
       <c r="C20" s="4"/>
@@ -1648,7 +1648,7 @@
       <c r="U20" s="26"/>
       <c r="V20" s="25"/>
     </row>
-    <row r="21" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="8"/>
       <c r="B21" s="6"/>
       <c r="C21" s="4"/>
@@ -1686,7 +1686,7 @@
       <c r="U21" s="26"/>
       <c r="V21" s="25"/>
     </row>
-    <row r="22" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="8"/>
       <c r="B22" s="6"/>
       <c r="C22" s="4"/>
@@ -1724,7 +1724,7 @@
       <c r="U22" s="26"/>
       <c r="V22" s="25"/>
     </row>
-    <row r="23" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="8"/>
       <c r="B23" s="6"/>
       <c r="C23" s="4"/>
@@ -1762,7 +1762,7 @@
       <c r="U23" s="26"/>
       <c r="V23" s="25"/>
     </row>
-    <row r="24" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="8"/>
       <c r="B24" s="6"/>
       <c r="C24" s="4"/>
@@ -1800,7 +1800,7 @@
       <c r="U24" s="26"/>
       <c r="V24" s="25"/>
     </row>
-    <row r="25" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="8"/>
       <c r="B25" s="6"/>
       <c r="C25" s="4"/>
@@ -1838,7 +1838,7 @@
       <c r="U25" s="26"/>
       <c r="V25" s="25"/>
     </row>
-    <row r="26" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="8"/>
       <c r="B26" s="6"/>
       <c r="C26" s="4"/>
@@ -1876,7 +1876,7 @@
       <c r="U26" s="26"/>
       <c r="V26" s="25"/>
     </row>
-    <row r="27" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="8"/>
       <c r="B27" s="6"/>
       <c r="C27" s="4"/>
@@ -1914,7 +1914,7 @@
       <c r="U27" s="26"/>
       <c r="V27" s="25"/>
     </row>
-    <row r="28" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="8"/>
       <c r="B28" s="6"/>
       <c r="C28" s="4"/>
@@ -1952,7 +1952,7 @@
       <c r="U28" s="26"/>
       <c r="V28" s="25"/>
     </row>
-    <row r="29" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="8"/>
       <c r="B29" s="6"/>
       <c r="C29" s="4"/>
@@ -1990,7 +1990,7 @@
       <c r="U29" s="26"/>
       <c r="V29" s="25"/>
     </row>
-    <row r="30" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="8"/>
       <c r="B30" s="6"/>
       <c r="C30" s="4"/>
@@ -2028,7 +2028,7 @@
       <c r="U30" s="26"/>
       <c r="V30" s="25"/>
     </row>
-    <row r="31" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="8"/>
       <c r="B31" s="6"/>
       <c r="C31" s="4"/>
@@ -2066,7 +2066,7 @@
       <c r="U31" s="26"/>
       <c r="V31" s="25"/>
     </row>
-    <row r="32" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="8"/>
       <c r="B32" s="6"/>
       <c r="C32" s="4"/>
@@ -2104,7 +2104,7 @@
       <c r="U32" s="26"/>
       <c r="V32" s="25"/>
     </row>
-    <row r="33" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="8"/>
       <c r="B33" s="6"/>
       <c r="C33" s="4"/>
@@ -2142,7 +2142,7 @@
       <c r="U33" s="26"/>
       <c r="V33" s="25"/>
     </row>
-    <row r="34" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="8"/>
       <c r="B34" s="6"/>
       <c r="C34" s="4"/>
@@ -2180,7 +2180,7 @@
       <c r="U34" s="26"/>
       <c r="V34" s="25"/>
     </row>
-    <row r="35" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="8"/>
       <c r="B35" s="6"/>
       <c r="C35" s="4"/>
@@ -2218,7 +2218,7 @@
       <c r="U35" s="26"/>
       <c r="V35" s="25"/>
     </row>
-    <row r="36" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="8"/>
       <c r="B36" s="6"/>
       <c r="C36" s="4"/>
@@ -2256,7 +2256,7 @@
       <c r="U36" s="26"/>
       <c r="V36" s="25"/>
     </row>
-    <row r="37" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="8"/>
       <c r="B37" s="6"/>
       <c r="C37" s="4"/>
@@ -2280,7 +2280,7 @@
       <c r="U37" s="26"/>
       <c r="V37" s="25"/>
     </row>
-    <row r="38" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="8"/>
       <c r="B38" s="6"/>
       <c r="C38" s="4"/>
@@ -2304,7 +2304,7 @@
       <c r="U38" s="26"/>
       <c r="V38" s="25"/>
     </row>
-    <row r="39" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="8"/>
       <c r="B39" s="6"/>
       <c r="C39" s="4"/>
@@ -2328,7 +2328,7 @@
       <c r="U39" s="26"/>
       <c r="V39" s="25"/>
     </row>
-    <row r="40" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="8"/>
       <c r="B40" s="6"/>
       <c r="C40" s="4"/>
@@ -2352,7 +2352,7 @@
       <c r="U40" s="26"/>
       <c r="V40" s="25"/>
     </row>
-    <row r="41" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="8"/>
       <c r="B41" s="6"/>
       <c r="C41" s="4"/>
@@ -2376,7 +2376,7 @@
       <c r="U41" s="26"/>
       <c r="V41" s="25"/>
     </row>
-    <row r="42" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="8"/>
       <c r="B42" s="6"/>
       <c r="C42" s="4"/>
@@ -2400,7 +2400,7 @@
       <c r="U42" s="26"/>
       <c r="V42" s="25"/>
     </row>
-    <row r="43" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="8"/>
       <c r="B43" s="6"/>
       <c r="C43" s="4"/>
@@ -2424,7 +2424,7 @@
       <c r="U43" s="26"/>
       <c r="V43" s="25"/>
     </row>
-    <row r="44" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="8"/>
       <c r="B44" s="6"/>
       <c r="C44" s="4"/>
@@ -2448,7 +2448,7 @@
       <c r="U44" s="26"/>
       <c r="V44" s="25"/>
     </row>
-    <row r="45" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="8"/>
       <c r="B45" s="6"/>
       <c r="C45" s="4"/>
@@ -2472,7 +2472,7 @@
       <c r="U45" s="26"/>
       <c r="V45" s="25"/>
     </row>
-    <row r="46" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="8"/>
       <c r="B46" s="6"/>
       <c r="C46" s="4"/>
@@ -2496,7 +2496,7 @@
       <c r="U46" s="26"/>
       <c r="V46" s="25"/>
     </row>
-    <row r="47" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="8"/>
       <c r="B47" s="6"/>
       <c r="C47" s="4"/>
@@ -2520,7 +2520,7 @@
       <c r="U47" s="26"/>
       <c r="V47" s="25"/>
     </row>
-    <row r="48" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="8"/>
       <c r="B48" s="6"/>
       <c r="C48" s="4"/>
@@ -2544,7 +2544,7 @@
       <c r="U48" s="26"/>
       <c r="V48" s="25"/>
     </row>
-    <row r="49" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="8"/>
       <c r="B49" s="6"/>
       <c r="C49" s="4"/>
@@ -2568,7 +2568,7 @@
       <c r="U49" s="26"/>
       <c r="V49" s="25"/>
     </row>
-    <row r="50" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="8"/>
       <c r="B50" s="6"/>
       <c r="C50" s="4"/>
@@ -2592,7 +2592,7 @@
       <c r="U50" s="26"/>
       <c r="V50" s="25"/>
     </row>
-    <row r="51" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="8"/>
       <c r="B51" s="6"/>
       <c r="C51" s="4"/>
@@ -2616,7 +2616,7 @@
       <c r="U51" s="26"/>
       <c r="V51" s="25"/>
     </row>
-    <row r="52" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="8"/>
       <c r="B52" s="6"/>
       <c r="C52" s="4"/>
@@ -2640,7 +2640,7 @@
       <c r="U52" s="26"/>
       <c r="V52" s="25"/>
     </row>
-    <row r="53" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="8"/>
       <c r="B53" s="6"/>
       <c r="C53" s="4"/>
@@ -2664,7 +2664,7 @@
       <c r="U53" s="26"/>
       <c r="V53" s="25"/>
     </row>
-    <row r="54" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="8"/>
       <c r="B54" s="6"/>
       <c r="C54" s="4"/>
@@ -2688,7 +2688,7 @@
       <c r="U54" s="26"/>
       <c r="V54" s="25"/>
     </row>
-    <row r="55" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="8"/>
       <c r="B55" s="6"/>
       <c r="C55" s="4"/>
@@ -2712,7 +2712,7 @@
       <c r="U55" s="26"/>
       <c r="V55" s="25"/>
     </row>
-    <row r="56" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="8"/>
       <c r="B56" s="6"/>
       <c r="C56" s="4"/>
@@ -2736,7 +2736,7 @@
       <c r="U56" s="26"/>
       <c r="V56" s="25"/>
     </row>
-    <row r="57" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="8"/>
       <c r="B57" s="6"/>
       <c r="C57" s="4"/>
@@ -2760,7 +2760,7 @@
       <c r="U57" s="26"/>
       <c r="V57" s="25"/>
     </row>
-    <row r="58" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="8"/>
       <c r="B58" s="6"/>
       <c r="C58" s="4"/>
@@ -2784,7 +2784,7 @@
       <c r="U58" s="26"/>
       <c r="V58" s="25"/>
     </row>
-    <row r="59" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="8"/>
       <c r="B59" s="6"/>
       <c r="C59" s="4"/>
@@ -2808,7 +2808,7 @@
       <c r="U59" s="26"/>
       <c r="V59" s="25"/>
     </row>
-    <row r="60" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="8"/>
       <c r="B60" s="6"/>
       <c r="C60" s="4"/>
@@ -2832,7 +2832,7 @@
       <c r="U60" s="26"/>
       <c r="V60" s="25"/>
     </row>
-    <row r="61" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="8"/>
       <c r="B61" s="6"/>
       <c r="C61" s="4"/>
@@ -2856,7 +2856,7 @@
       <c r="U61" s="26"/>
       <c r="V61" s="25"/>
     </row>
-    <row r="62" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="8"/>
       <c r="B62" s="6"/>
       <c r="C62" s="4"/>
@@ -2880,7 +2880,7 @@
       <c r="U62" s="26"/>
       <c r="V62" s="25"/>
     </row>
-    <row r="63" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="8"/>
       <c r="B63" s="6"/>
       <c r="C63" s="4"/>
@@ -2904,7 +2904,7 @@
       <c r="U63" s="26"/>
       <c r="V63" s="25"/>
     </row>
-    <row r="64" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="8"/>
       <c r="B64" s="6"/>
       <c r="C64" s="4"/>
@@ -2928,7 +2928,7 @@
       <c r="U64" s="26"/>
       <c r="V64" s="25"/>
     </row>
-    <row r="65" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="8"/>
       <c r="B65" s="6"/>
       <c r="C65" s="4"/>
@@ -2952,7 +2952,7 @@
       <c r="U65" s="26"/>
       <c r="V65" s="25"/>
     </row>
-    <row r="66" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="8"/>
       <c r="B66" s="6"/>
       <c r="C66" s="4"/>
@@ -2976,7 +2976,7 @@
       <c r="U66" s="26"/>
       <c r="V66" s="25"/>
     </row>
-    <row r="67" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="8"/>
       <c r="B67" s="6"/>
       <c r="C67" s="4"/>
@@ -3000,7 +3000,7 @@
       <c r="U67" s="26"/>
       <c r="V67" s="25"/>
     </row>
-    <row r="68" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="8"/>
       <c r="B68" s="6"/>
       <c r="C68" s="4"/>
@@ -3024,7 +3024,7 @@
       <c r="U68" s="26"/>
       <c r="V68" s="25"/>
     </row>
-    <row r="69" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="8"/>
       <c r="B69" s="6"/>
       <c r="C69" s="4"/>
@@ -3048,7 +3048,7 @@
       <c r="U69" s="26"/>
       <c r="V69" s="25"/>
     </row>
-    <row r="70" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="8"/>
       <c r="B70" s="6"/>
       <c r="C70" s="4"/>
@@ -3072,7 +3072,7 @@
       <c r="U70" s="26"/>
       <c r="V70" s="25"/>
     </row>
-    <row r="71" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="8"/>
       <c r="B71" s="6"/>
       <c r="C71" s="4"/>
@@ -3096,7 +3096,7 @@
       <c r="U71" s="26"/>
       <c r="V71" s="25"/>
     </row>
-    <row r="72" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="8"/>
       <c r="B72" s="6"/>
       <c r="C72" s="4"/>
@@ -3120,7 +3120,7 @@
       <c r="U72" s="26"/>
       <c r="V72" s="25"/>
     </row>
-    <row r="73" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="8"/>
       <c r="B73" s="6"/>
       <c r="C73" s="4"/>
@@ -3144,7 +3144,7 @@
       <c r="U73" s="26"/>
       <c r="V73" s="25"/>
     </row>
-    <row r="74" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="8"/>
       <c r="B74" s="6"/>
       <c r="C74" s="4"/>
@@ -3168,7 +3168,7 @@
       <c r="U74" s="26"/>
       <c r="V74" s="25"/>
     </row>
-    <row r="75" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="8"/>
       <c r="B75" s="6"/>
       <c r="C75" s="4"/>
@@ -3192,7 +3192,7 @@
       <c r="U75" s="26"/>
       <c r="V75" s="25"/>
     </row>
-    <row r="76" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="8"/>
       <c r="B76" s="6"/>
       <c r="C76" s="4"/>
@@ -3216,7 +3216,7 @@
       <c r="U76" s="26"/>
       <c r="V76" s="25"/>
     </row>
-    <row r="77" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="8"/>
       <c r="B77" s="6"/>
       <c r="C77" s="4"/>
@@ -3240,7 +3240,7 @@
       <c r="U77" s="26"/>
       <c r="V77" s="25"/>
     </row>
-    <row r="78" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="8"/>
       <c r="B78" s="6"/>
       <c r="C78" s="4"/>
@@ -3264,7 +3264,7 @@
       <c r="U78" s="26"/>
       <c r="V78" s="25"/>
     </row>
-    <row r="79" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="8"/>
       <c r="B79" s="6"/>
       <c r="C79" s="4"/>
@@ -3288,7 +3288,7 @@
       <c r="U79" s="26"/>
       <c r="V79" s="25"/>
     </row>
-    <row r="80" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="8"/>
       <c r="B80" s="6"/>
       <c r="C80" s="4"/>
@@ -3312,7 +3312,7 @@
       <c r="U80" s="26"/>
       <c r="V80" s="25"/>
     </row>
-    <row r="81" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="8"/>
       <c r="B81" s="6"/>
       <c r="C81" s="4"/>
@@ -3336,7 +3336,7 @@
       <c r="U81" s="26"/>
       <c r="V81" s="25"/>
     </row>
-    <row r="82" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="8"/>
       <c r="B82" s="6"/>
       <c r="C82" s="4"/>
@@ -3360,7 +3360,7 @@
       <c r="U82" s="26"/>
       <c r="V82" s="25"/>
     </row>
-    <row r="83" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="8"/>
       <c r="B83" s="6"/>
       <c r="C83" s="4"/>
@@ -3384,7 +3384,7 @@
       <c r="U83" s="26"/>
       <c r="V83" s="25"/>
     </row>
-    <row r="84" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="8"/>
       <c r="B84" s="6"/>
       <c r="C84" s="4"/>
@@ -3408,7 +3408,7 @@
       <c r="U84" s="26"/>
       <c r="V84" s="25"/>
     </row>
-    <row r="85" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="8"/>
       <c r="B85" s="6"/>
       <c r="C85" s="4"/>
@@ -3432,7 +3432,7 @@
       <c r="U85" s="26"/>
       <c r="V85" s="25"/>
     </row>
-    <row r="86" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="8"/>
       <c r="B86" s="6"/>
       <c r="C86" s="4"/>
@@ -3456,7 +3456,7 @@
       <c r="U86" s="26"/>
       <c r="V86" s="25"/>
     </row>
-    <row r="87" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="8"/>
       <c r="B87" s="6"/>
       <c r="C87" s="4"/>
@@ -3480,7 +3480,7 @@
       <c r="U87" s="26"/>
       <c r="V87" s="25"/>
     </row>
-    <row r="88" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="8"/>
       <c r="B88" s="6"/>
       <c r="C88" s="4"/>
@@ -3504,7 +3504,7 @@
       <c r="U88" s="26"/>
       <c r="V88" s="25"/>
     </row>
-    <row r="89" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="8"/>
       <c r="B89" s="6"/>
       <c r="C89" s="4"/>
@@ -3528,7 +3528,7 @@
       <c r="U89" s="26"/>
       <c r="V89" s="25"/>
     </row>
-    <row r="90" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="8"/>
       <c r="B90" s="6"/>
       <c r="C90" s="4"/>
@@ -3552,7 +3552,7 @@
       <c r="U90" s="26"/>
       <c r="V90" s="25"/>
     </row>
-    <row r="91" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="8"/>
       <c r="B91" s="6"/>
       <c r="C91" s="4"/>
@@ -3576,7 +3576,7 @@
       <c r="U91" s="26"/>
       <c r="V91" s="25"/>
     </row>
-    <row r="92" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="8"/>
       <c r="B92" s="6"/>
       <c r="C92" s="4"/>
@@ -3600,7 +3600,7 @@
       <c r="U92" s="26"/>
       <c r="V92" s="25"/>
     </row>
-    <row r="93" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="8"/>
       <c r="B93" s="6"/>
       <c r="C93" s="4"/>
@@ -3624,7 +3624,7 @@
       <c r="U93" s="26"/>
       <c r="V93" s="25"/>
     </row>
-    <row r="94" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="8"/>
       <c r="B94" s="6"/>
       <c r="C94" s="4"/>
@@ -3648,7 +3648,7 @@
       <c r="U94" s="26"/>
       <c r="V94" s="25"/>
     </row>
-    <row r="95" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="8"/>
       <c r="B95" s="6"/>
       <c r="C95" s="4"/>
@@ -3672,7 +3672,7 @@
       <c r="U95" s="26"/>
       <c r="V95" s="25"/>
     </row>
-    <row r="96" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="8"/>
       <c r="B96" s="6"/>
       <c r="C96" s="4"/>
@@ -3696,7 +3696,7 @@
       <c r="U96" s="26"/>
       <c r="V96" s="25"/>
     </row>
-    <row r="97" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="8"/>
       <c r="B97" s="6"/>
       <c r="C97" s="4"/>
@@ -3720,7 +3720,7 @@
       <c r="U97" s="26"/>
       <c r="V97" s="25"/>
     </row>
-    <row r="98" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="8"/>
       <c r="B98" s="6"/>
       <c r="C98" s="4"/>
@@ -3744,7 +3744,7 @@
       <c r="U98" s="26"/>
       <c r="V98" s="25"/>
     </row>
-    <row r="99" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="8"/>
       <c r="B99" s="6"/>
       <c r="C99" s="4"/>
@@ -3768,7 +3768,7 @@
       <c r="U99" s="26"/>
       <c r="V99" s="25"/>
     </row>
-    <row r="100" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="8"/>
       <c r="B100" s="6"/>
       <c r="C100" s="4"/>
@@ -3792,7 +3792,7 @@
       <c r="U100" s="26"/>
       <c r="V100" s="25"/>
     </row>
-    <row r="101" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="8"/>
       <c r="B101" s="6"/>
       <c r="C101" s="4"/>
@@ -3816,7 +3816,7 @@
       <c r="U101" s="26"/>
       <c r="V101" s="25"/>
     </row>
-    <row r="102" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="8"/>
       <c r="B102" s="6"/>
       <c r="C102" s="4"/>
@@ -3840,7 +3840,7 @@
       <c r="U102" s="26"/>
       <c r="V102" s="25"/>
     </row>
-    <row r="103" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="8"/>
       <c r="B103" s="6"/>
       <c r="C103" s="4"/>
@@ -3864,7 +3864,7 @@
       <c r="U103" s="26"/>
       <c r="V103" s="25"/>
     </row>
-    <row r="104" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="8"/>
       <c r="B104" s="6"/>
       <c r="C104" s="4"/>
@@ -3888,7 +3888,7 @@
       <c r="U104" s="26"/>
       <c r="V104" s="25"/>
     </row>
-    <row r="105" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="8"/>
       <c r="B105" s="6"/>
       <c r="C105" s="4"/>
@@ -3912,7 +3912,7 @@
       <c r="U105" s="26"/>
       <c r="V105" s="25"/>
     </row>
-    <row r="106" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="8"/>
       <c r="B106" s="6"/>
       <c r="C106" s="4"/>
@@ -3936,7 +3936,7 @@
       <c r="U106" s="26"/>
       <c r="V106" s="25"/>
     </row>
-    <row r="107" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="8"/>
       <c r="B107" s="6"/>
       <c r="C107" s="4"/>
@@ -3960,7 +3960,7 @@
       <c r="U107" s="26"/>
       <c r="V107" s="25"/>
     </row>
-    <row r="108" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="8"/>
       <c r="B108" s="6"/>
       <c r="C108" s="4"/>
@@ -3984,7 +3984,7 @@
       <c r="U108" s="26"/>
       <c r="V108" s="25"/>
     </row>
-    <row r="109" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="8"/>
       <c r="B109" s="6"/>
       <c r="C109" s="4"/>
@@ -4008,7 +4008,7 @@
       <c r="U109" s="26"/>
       <c r="V109" s="25"/>
     </row>
-    <row r="110" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="8"/>
       <c r="B110" s="6"/>
       <c r="C110" s="4"/>
@@ -4032,7 +4032,7 @@
       <c r="U110" s="26"/>
       <c r="V110" s="25"/>
     </row>
-    <row r="111" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="8"/>
       <c r="B111" s="6"/>
       <c r="C111" s="4"/>
@@ -4056,7 +4056,7 @@
       <c r="U111" s="26"/>
       <c r="V111" s="25"/>
     </row>
-    <row r="112" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="8"/>
       <c r="B112" s="6"/>
       <c r="C112" s="4"/>
@@ -4080,7 +4080,7 @@
       <c r="U112" s="26"/>
       <c r="V112" s="25"/>
     </row>
-    <row r="113" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="8"/>
       <c r="B113" s="6"/>
       <c r="C113" s="4"/>
@@ -4104,7 +4104,7 @@
       <c r="U113" s="26"/>
       <c r="V113" s="25"/>
     </row>
-    <row r="114" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="8"/>
       <c r="B114" s="6"/>
       <c r="C114" s="4"/>
@@ -4128,7 +4128,7 @@
       <c r="U114" s="26"/>
       <c r="V114" s="25"/>
     </row>
-    <row r="115" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="8"/>
       <c r="B115" s="6"/>
       <c r="C115" s="4"/>
@@ -4152,7 +4152,7 @@
       <c r="U115" s="26"/>
       <c r="V115" s="25"/>
     </row>
-    <row r="116" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="8"/>
       <c r="B116" s="6"/>
       <c r="C116" s="4"/>
@@ -4176,7 +4176,7 @@
       <c r="U116" s="26"/>
       <c r="V116" s="25"/>
     </row>
-    <row r="117" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="8"/>
       <c r="B117" s="6"/>
       <c r="C117" s="4"/>
@@ -4200,7 +4200,7 @@
       <c r="U117" s="26"/>
       <c r="V117" s="25"/>
     </row>
-    <row r="118" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="8"/>
       <c r="B118" s="6"/>
       <c r="C118" s="4"/>
@@ -4224,7 +4224,7 @@
       <c r="U118" s="26"/>
       <c r="V118" s="25"/>
     </row>
-    <row r="119" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="8"/>
       <c r="B119" s="6"/>
       <c r="C119" s="4"/>
@@ -4248,7 +4248,7 @@
       <c r="U119" s="26"/>
       <c r="V119" s="25"/>
     </row>
-    <row r="120" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="8"/>
       <c r="B120" s="6"/>
       <c r="C120" s="4"/>
@@ -4272,7 +4272,7 @@
       <c r="U120" s="26"/>
       <c r="V120" s="25"/>
     </row>
-    <row r="121" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="8"/>
       <c r="B121" s="6"/>
       <c r="C121" s="4"/>
@@ -4296,7 +4296,7 @@
       <c r="U121" s="26"/>
       <c r="V121" s="25"/>
     </row>
-    <row r="122" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="8"/>
       <c r="B122" s="6"/>
       <c r="C122" s="4"/>
@@ -4320,7 +4320,7 @@
       <c r="U122" s="26"/>
       <c r="V122" s="25"/>
     </row>
-    <row r="123" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="8"/>
       <c r="B123" s="6"/>
       <c r="C123" s="4"/>
@@ -4344,7 +4344,7 @@
       <c r="U123" s="26"/>
       <c r="V123" s="25"/>
     </row>
-    <row r="124" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="8"/>
       <c r="B124" s="6"/>
       <c r="C124" s="4"/>
@@ -4368,7 +4368,7 @@
       <c r="U124" s="26"/>
       <c r="V124" s="25"/>
     </row>
-    <row r="125" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="8"/>
       <c r="B125" s="6"/>
       <c r="C125" s="4"/>
@@ -4392,7 +4392,7 @@
       <c r="U125" s="26"/>
       <c r="V125" s="25"/>
     </row>
-    <row r="126" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="8"/>
       <c r="B126" s="6"/>
       <c r="C126" s="4"/>
@@ -4416,7 +4416,7 @@
       <c r="U126" s="26"/>
       <c r="V126" s="25"/>
     </row>
-    <row r="127" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="8"/>
       <c r="B127" s="6"/>
       <c r="C127" s="4"/>
@@ -4440,7 +4440,7 @@
       <c r="U127" s="26"/>
       <c r="V127" s="25"/>
     </row>
-    <row r="128" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="8"/>
       <c r="B128" s="6"/>
       <c r="C128" s="4"/>
@@ -4464,7 +4464,7 @@
       <c r="U128" s="26"/>
       <c r="V128" s="25"/>
     </row>
-    <row r="129" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="8"/>
       <c r="B129" s="6"/>
       <c r="C129" s="4"/>
@@ -4488,7 +4488,7 @@
       <c r="U129" s="26"/>
       <c r="V129" s="25"/>
     </row>
-    <row r="130" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="8"/>
       <c r="B130" s="6"/>
       <c r="C130" s="4"/>
@@ -4512,7 +4512,7 @@
       <c r="U130" s="26"/>
       <c r="V130" s="25"/>
     </row>
-    <row r="131" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="8"/>
       <c r="B131" s="6"/>
       <c r="C131" s="4"/>
@@ -4536,7 +4536,7 @@
       <c r="U131" s="26"/>
       <c r="V131" s="25"/>
     </row>
-    <row r="132" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="8"/>
       <c r="B132" s="6"/>
       <c r="C132" s="4"/>
@@ -4560,7 +4560,7 @@
       <c r="U132" s="26"/>
       <c r="V132" s="25"/>
     </row>
-    <row r="133" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="8"/>
       <c r="B133" s="6"/>
       <c r="C133" s="4"/>
@@ -4584,7 +4584,7 @@
       <c r="U133" s="26"/>
       <c r="V133" s="25"/>
     </row>
-    <row r="134" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="8"/>
       <c r="B134" s="6"/>
       <c r="C134" s="4"/>
@@ -4608,7 +4608,7 @@
       <c r="U134" s="26"/>
       <c r="V134" s="25"/>
     </row>
-    <row r="135" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="8"/>
       <c r="B135" s="6"/>
       <c r="C135" s="4"/>
@@ -4632,7 +4632,7 @@
       <c r="U135" s="26"/>
       <c r="V135" s="25"/>
     </row>
-    <row r="136" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="8"/>
       <c r="B136" s="6"/>
       <c r="C136" s="4"/>
@@ -4656,7 +4656,7 @@
       <c r="U136" s="26"/>
       <c r="V136" s="25"/>
     </row>
-    <row r="137" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="8"/>
       <c r="B137" s="6"/>
       <c r="C137" s="4"/>
@@ -4680,7 +4680,7 @@
       <c r="U137" s="26"/>
       <c r="V137" s="25"/>
     </row>
-    <row r="138" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="8"/>
       <c r="B138" s="6"/>
       <c r="C138" s="4"/>
@@ -4704,7 +4704,7 @@
       <c r="U138" s="26"/>
       <c r="V138" s="25"/>
     </row>
-    <row r="139" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="8"/>
       <c r="B139" s="6"/>
       <c r="C139" s="4"/>
@@ -4728,7 +4728,7 @@
       <c r="U139" s="26"/>
       <c r="V139" s="25"/>
     </row>
-    <row r="140" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="8"/>
       <c r="B140" s="6"/>
       <c r="C140" s="4"/>
@@ -4752,7 +4752,7 @@
       <c r="U140" s="26"/>
       <c r="V140" s="25"/>
     </row>
-    <row r="141" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="8"/>
       <c r="B141" s="6"/>
       <c r="C141" s="4"/>
@@ -4776,7 +4776,7 @@
       <c r="U141" s="26"/>
       <c r="V141" s="25"/>
     </row>
-    <row r="142" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="8"/>
       <c r="B142" s="6"/>
       <c r="C142" s="4"/>
@@ -4800,7 +4800,7 @@
       <c r="U142" s="26"/>
       <c r="V142" s="25"/>
     </row>
-    <row r="143" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="8"/>
       <c r="B143" s="6"/>
       <c r="C143" s="4"/>
@@ -4824,7 +4824,7 @@
       <c r="U143" s="26"/>
       <c r="V143" s="25"/>
     </row>
-    <row r="144" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="8"/>
       <c r="B144" s="6"/>
       <c r="C144" s="4"/>
@@ -4848,7 +4848,7 @@
       <c r="U144" s="26"/>
       <c r="V144" s="25"/>
     </row>
-    <row r="145" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="8"/>
       <c r="B145" s="6"/>
       <c r="C145" s="4"/>
@@ -4872,7 +4872,7 @@
       <c r="U145" s="26"/>
       <c r="V145" s="25"/>
     </row>
-    <row r="146" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="8"/>
       <c r="B146" s="6"/>
       <c r="C146" s="4"/>
@@ -4896,7 +4896,7 @@
       <c r="U146" s="26"/>
       <c r="V146" s="25"/>
     </row>
-    <row r="147" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="8"/>
       <c r="B147" s="6"/>
       <c r="C147" s="4"/>
@@ -4920,7 +4920,7 @@
       <c r="U147" s="26"/>
       <c r="V147" s="25"/>
     </row>
-    <row r="148" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="8"/>
       <c r="B148" s="6"/>
       <c r="C148" s="4"/>
@@ -4944,7 +4944,7 @@
       <c r="U148" s="26"/>
       <c r="V148" s="25"/>
     </row>
-    <row r="149" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="8"/>
       <c r="B149" s="6"/>
       <c r="C149" s="4"/>
@@ -4968,7 +4968,7 @@
       <c r="U149" s="26"/>
       <c r="V149" s="25"/>
     </row>
-    <row r="150" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="8"/>
       <c r="B150" s="6"/>
       <c r="C150" s="4"/>
@@ -4992,7 +4992,7 @@
       <c r="U150" s="26"/>
       <c r="V150" s="25"/>
     </row>
-    <row r="151" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="8"/>
       <c r="B151" s="6"/>
       <c r="C151" s="4"/>
@@ -5016,7 +5016,7 @@
       <c r="U151" s="26"/>
       <c r="V151" s="25"/>
     </row>
-    <row r="152" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="8"/>
       <c r="B152" s="6"/>
       <c r="C152" s="4"/>
@@ -5040,7 +5040,7 @@
       <c r="U152" s="26"/>
       <c r="V152" s="25"/>
     </row>
-    <row r="153" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="8"/>
       <c r="B153" s="6"/>
       <c r="C153" s="4"/>
@@ -5064,7 +5064,7 @@
       <c r="U153" s="26"/>
       <c r="V153" s="25"/>
     </row>
-    <row r="154" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="8"/>
       <c r="B154" s="6"/>
       <c r="C154" s="4"/>
@@ -5088,7 +5088,7 @@
       <c r="U154" s="26"/>
       <c r="V154" s="25"/>
     </row>
-    <row r="155" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="8"/>
       <c r="B155" s="6"/>
       <c r="C155" s="4"/>
@@ -5112,7 +5112,7 @@
       <c r="U155" s="26"/>
       <c r="V155" s="25"/>
     </row>
-    <row r="156" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="8"/>
       <c r="B156" s="6"/>
       <c r="C156" s="4"/>
@@ -5136,7 +5136,7 @@
       <c r="U156" s="26"/>
       <c r="V156" s="25"/>
     </row>
-    <row r="157" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="8"/>
       <c r="B157" s="6"/>
       <c r="C157" s="4"/>
@@ -5160,7 +5160,7 @@
       <c r="U157" s="26"/>
       <c r="V157" s="25"/>
     </row>
-    <row r="158" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="8"/>
       <c r="B158" s="6"/>
       <c r="C158" s="4"/>
@@ -5184,7 +5184,7 @@
       <c r="U158" s="26"/>
       <c r="V158" s="25"/>
     </row>
-    <row r="159" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="8"/>
       <c r="B159" s="6"/>
       <c r="C159" s="4"/>
@@ -5208,7 +5208,7 @@
       <c r="U159" s="26"/>
       <c r="V159" s="25"/>
     </row>
-    <row r="160" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="8"/>
       <c r="B160" s="6"/>
       <c r="C160" s="4"/>
@@ -5232,7 +5232,7 @@
       <c r="U160" s="26"/>
       <c r="V160" s="25"/>
     </row>
-    <row r="161" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="8"/>
       <c r="B161" s="6"/>
       <c r="C161" s="4"/>
@@ -5256,7 +5256,7 @@
       <c r="U161" s="26"/>
       <c r="V161" s="25"/>
     </row>
-    <row r="162" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" s="8"/>
       <c r="B162" s="6"/>
       <c r="C162" s="4"/>
@@ -5280,7 +5280,7 @@
       <c r="U162" s="26"/>
       <c r="V162" s="25"/>
     </row>
-    <row r="163" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A163" s="8"/>
       <c r="B163" s="6"/>
       <c r="C163" s="4"/>
@@ -5304,7 +5304,7 @@
       <c r="U163" s="26"/>
       <c r="V163" s="25"/>
     </row>
-    <row r="164" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A164" s="8"/>
       <c r="B164" s="6"/>
       <c r="C164" s="4"/>
@@ -5328,7 +5328,7 @@
       <c r="U164" s="26"/>
       <c r="V164" s="25"/>
     </row>
-    <row r="165" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A165" s="8"/>
       <c r="B165" s="6"/>
       <c r="C165" s="4"/>
@@ -5352,7 +5352,7 @@
       <c r="U165" s="26"/>
       <c r="V165" s="25"/>
     </row>
-    <row r="166" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" s="8"/>
       <c r="B166" s="6"/>
       <c r="C166" s="4"/>
@@ -5376,7 +5376,7 @@
       <c r="U166" s="26"/>
       <c r="V166" s="25"/>
     </row>
-    <row r="167" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A167" s="8"/>
       <c r="B167" s="6"/>
       <c r="C167" s="4"/>
@@ -5400,7 +5400,7 @@
       <c r="U167" s="26"/>
       <c r="V167" s="25"/>
     </row>
-    <row r="168" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="Q168" s="25"/>
       <c r="R168" s="24"/>
       <c r="S168" s="26"/>
@@ -5408,7 +5408,7 @@
       <c r="U168" s="26"/>
       <c r="V168" s="25"/>
     </row>
-    <row r="169" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="Q169" s="25"/>
       <c r="R169" s="24"/>
       <c r="S169" s="26"/>
@@ -5416,7 +5416,7 @@
       <c r="U169" s="26"/>
       <c r="V169" s="25"/>
     </row>
-    <row r="170" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="Q170" s="25"/>
       <c r="R170" s="24"/>
       <c r="S170" s="26"/>
@@ -5424,7 +5424,7 @@
       <c r="U170" s="26"/>
       <c r="V170" s="25"/>
     </row>
-    <row r="171" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="Q171" s="25"/>
       <c r="R171" s="24"/>
       <c r="S171" s="26"/>
@@ -5432,7 +5432,7 @@
       <c r="U171" s="26"/>
       <c r="V171" s="25"/>
     </row>
-    <row r="172" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="Q172" s="25"/>
       <c r="R172" s="24"/>
       <c r="S172" s="26"/>
@@ -5440,7 +5440,7 @@
       <c r="U172" s="26"/>
       <c r="V172" s="25"/>
     </row>
-    <row r="173" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="Q173" s="25"/>
       <c r="R173" s="24"/>
       <c r="S173" s="26"/>
@@ -5448,7 +5448,7 @@
       <c r="U173" s="26"/>
       <c r="V173" s="25"/>
     </row>
-    <row r="174" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="Q174" s="25"/>
       <c r="R174" s="24"/>
       <c r="S174" s="26"/>
@@ -5456,7 +5456,7 @@
       <c r="U174" s="26"/>
       <c r="V174" s="25"/>
     </row>
-    <row r="175" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="Q175" s="25"/>
       <c r="R175" s="24"/>
       <c r="S175" s="26"/>
@@ -5464,7 +5464,7 @@
       <c r="U175" s="26"/>
       <c r="V175" s="25"/>
     </row>
-    <row r="176" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="Q176" s="25"/>
       <c r="R176" s="24"/>
       <c r="S176" s="26"/>
@@ -5472,7 +5472,7 @@
       <c r="U176" s="26"/>
       <c r="V176" s="25"/>
     </row>
-    <row r="177" spans="17:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="17:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="Q177" s="25"/>
       <c r="R177" s="24"/>
       <c r="S177" s="26"/>
@@ -5480,7 +5480,7 @@
       <c r="U177" s="26"/>
       <c r="V177" s="25"/>
     </row>
-    <row r="178" spans="17:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="17:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="Q178" s="25"/>
       <c r="R178" s="24"/>
       <c r="S178" s="26"/>
@@ -5488,7 +5488,7 @@
       <c r="U178" s="26"/>
       <c r="V178" s="25"/>
     </row>
-    <row r="179" spans="17:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="17:22" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="Q179" s="25"/>
       <c r="R179" s="24"/>
       <c r="S179" s="26"/>

</xml_diff>